<commit_message>
Rowgate run: contract tests and approved decisions
Four ACTIVE rows broken by feature/fast-checkout, each cited by the cell
that states the rule and covered by a test named after it:

  F1 Orders!C14  create must return 201                  -> fix code
  F2 Billing!E9  currency dropped from the invoice        -> record breaking change
  F3 Auth!E5     bad secret must be 401                   -> fix code
  F4 Errors!D6   the shared error envelope, not FastAPI's -> fix code
                 {"detail": ...}  (related: Auth!E5)

Two holds cleared: Orders!D11 (req_id keeps serialization_alias
"request_id", so the wire name is unchanged) and Orders!E5 ("pending" is
inside the allowed enum).

Three tests red -> green; F2 stays red and is recorded as breaking with
Billing!H9 = BREAKING and Changelog row 6.

The date in that Changelog row is a human edit, not Bob's: see
bob_sessions/README.md.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contract/api-contract.xlsx
+++ b/contract/api-contract.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,6 +157,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1893,7 +1894,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>BREAKING</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -2701,7 +2702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2847,6 +2848,38 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>v3.3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Billing!E9</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>currency field removed from GET /invoices/{id} response</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>breaking, accepted</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A. Okafor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>